<commit_message>
I have updated the assumptions to the table and explain the behaviour of them
</commit_message>
<xml_diff>
--- a/Formal/AHB_Lite_Verification_Table.xlsx
+++ b/Formal/AHB_Lite_Verification_Table.xlsx
@@ -5,10 +5,11 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="AHB-Lite Verification" sheetId="1" state="visible" r:id="rId2"/>
+    <sheet name="Sheet2" sheetId="2" state="visible" r:id="rId3"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -20,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="116">
   <si>
     <t xml:space="preserve">Assertion ID</t>
   </si>
@@ -110,6 +111,264 @@
   </si>
   <si>
     <t xml:space="preserve">Add exit condition to FSM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assumption ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reference Figure / Section</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Actionable Fix (TB Update)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">assume_reset_htrans</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unreachable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Asynchronous Reset: HTRANS initializes to IDLE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Section 7.1.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">None required (Expected Formal Behavior)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">assume_valid_htrans</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Transfer Validity: HTRANS restricted to legal values</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Section 3.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">assume_valid_hburst</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pass</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Burst Validity: HBURST restricted to 0-7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Section 3.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">assume_valid_hsize</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Size Validity: HSIZE restricted to 32-bit bounds</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Section 3.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">assume_valid_hwrite</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Signal Integrity: HWRITE has no X/Z states</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Section 3.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">assume_valid_hsel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Signal Integrity: HSEL has no X/Z states</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Section 4.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">assume_valid_hready</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Signal Integrity: HREADY has no X/Z states</t>
+  </si>
+  <si>
+    <t xml:space="preserve">assume_valid_haddr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Signal Integrity: HADDR valid during active transfer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">assume_align_halfword</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Address Alignment: Halfword aligned to 2-byte</t>
+  </si>
+  <si>
+    <t xml:space="preserve">assume_align_word</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Address Alignment: Word aligned to 4-byte</t>
+  </si>
+  <si>
+    <t xml:space="preserve">assume_1kb_boundary</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Boundary Limit: Bursts must not cross 1KB boundary</t>
+  </si>
+  <si>
+    <t xml:space="preserve">assume_stable_haddr_wait</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wait-State Stability: HADDR held during HREADY=0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">assume_stable_htrans_wait</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wait-State Stability: HTRANS held during HREADY=0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">assume_stable_hsize_wait</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wait-State Stability: HSIZE held during HREADY=0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">assume_stable_hburst_wait</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wait-State Stability: HBURST held during HREADY=0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">assume_stable_hwrite_wait</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wait-State Stability: HWRITE held during HREADY=0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">assume_stable_hsel_wait</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wait-State Stability: HSEL held during HREADY=0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">assume_no_seq_after_idle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Protocol Flow: SEQ cannot immediately follow IDLE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">assume_valid_seq_pred</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Protocol Flow: Valid predecessors for SEQ phase</t>
+  </si>
+  <si>
+    <t xml:space="preserve">assume_valid_busy_pred</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Protocol Flow: Valid predecessors for BUSY phase</t>
+  </si>
+  <si>
+    <t xml:space="preserve">assume_single_no_seq</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Protocol Flow: SINGLE burst forbids SEQ transfers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">assume_single_no_busy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Protocol Flow: SINGLE burst forbids BUSY transfers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">assume_const_hsize_burst</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Burst Integrity: Constant HSIZE during burst</t>
+  </si>
+  <si>
+    <t xml:space="preserve">assume_const_hwrite_burst</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Burst Integrity: Constant HWRITE during burst</t>
+  </si>
+  <si>
+    <t xml:space="preserve">assume_const_hburst_burst</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Burst Integrity: Constant HBURST during burst</t>
+  </si>
+  <si>
+    <t xml:space="preserve">assume_burst_len_incr4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Burst Length: INCR4 executes exactly 4 beats</t>
+  </si>
+  <si>
+    <t xml:space="preserve">assume_burst_len_wrap4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Burst Length: WRAP4 executes exactly 4 beats</t>
+  </si>
+  <si>
+    <t xml:space="preserve">assume_burst_len_incr8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Burst Length: INCR8 executes exactly 8 beats</t>
+  </si>
+  <si>
+    <t xml:space="preserve">assume_burst_len_wrap8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Burst Length: WRAP8 executes exactly 8 beats</t>
+  </si>
+  <si>
+    <t xml:space="preserve">assume_burst_len_incr16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Burst Length: INCR16 executes exactly 16 beats</t>
+  </si>
+  <si>
+    <t xml:space="preserve">assume_burst_len_wrap16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Burst Length: WRAP16 executes exactly 16 beats</t>
+  </si>
+  <si>
+    <t xml:space="preserve">assume_incr_addr_math</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Burst Address: INCR strictly increments by HSIZE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">assume_busy_addr_stable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Protocol Flow: BUSY phase maintains stable address</t>
+  </si>
+  <si>
+    <t xml:space="preserve">assume_wrap4_word_bound</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Burst Boundary: WRAP4 respects 16-byte wrap limit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">assume_wrap8_word_bound</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Burst Boundary: WRAP8 respects 32-byte wrap limit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">assume_wrap16_word_bound</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Burst Boundary: WRAP16 respects 64-byte wrap limit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">assume_wrap4_hw_bound</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Burst Boundary: WRAP4 Halfword respects 8-byte limit</t>
   </si>
 </sst>
 </file>
@@ -120,7 +379,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0.00"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -166,13 +425,42 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <color rgb="FF000040"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <color rgb="FF2BD0D2"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF2BD0D2"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00FF00"/>
+        <bgColor rgb="FF2BD0D2"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -209,7 +497,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="10">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -227,6 +515,26 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -251,7 +559,7 @@
       <rgbColor rgb="FF00FFFF"/>
       <rgbColor rgb="FF800000"/>
       <rgbColor rgb="FF008000"/>
-      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FF000040"/>
       <rgbColor rgb="FF808000"/>
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF008080"/>
@@ -282,7 +590,7 @@
       <rgbColor rgb="FFCC99FF"/>
       <rgbColor rgb="FFFFCC99"/>
       <rgbColor rgb="FF3366FF"/>
-      <rgbColor rgb="FF33CCCC"/>
+      <rgbColor rgb="FF2BD0D2"/>
       <rgbColor rgb="FF99CC00"/>
       <rgbColor rgb="FFFFCC00"/>
       <rgbColor rgb="FFFF9900"/>
@@ -314,7 +622,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="17.09"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="47.52"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="31.81"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="37.1"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="37.11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1025" min="6" style="0" width="8.67"/>
   </cols>
   <sheetData>
@@ -450,4 +758,676 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:E38"/>
+  <sheetFormatPr defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="27.55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12.13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="47.56"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="24.07"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="36.99"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="C2" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="D2" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="E2" s="0" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="D3" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="E3" s="0" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="C4" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="D4" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="E4" s="0" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="D5" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="E5" s="0" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" s="0" t="s">
+        <v>49</v>
+      </c>
+      <c r="D6" s="0" t="s">
+        <v>50</v>
+      </c>
+      <c r="E6" s="0" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C7" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="D7" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="E7" s="0" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C8" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="D8" s="0" t="s">
+        <v>50</v>
+      </c>
+      <c r="E8" s="0" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9" s="0" t="s">
+        <v>57</v>
+      </c>
+      <c r="D9" s="0" t="s">
+        <v>50</v>
+      </c>
+      <c r="E9" s="0" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C10" s="0" t="s">
+        <v>59</v>
+      </c>
+      <c r="D10" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="E10" s="0" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C11" s="0" t="s">
+        <v>61</v>
+      </c>
+      <c r="D11" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="E11" s="0" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="B12" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" s="0" t="s">
+        <v>63</v>
+      </c>
+      <c r="D12" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="E12" s="0" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C13" s="0" t="s">
+        <v>65</v>
+      </c>
+      <c r="D13" s="0" t="s">
+        <v>50</v>
+      </c>
+      <c r="E13" s="0" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C14" s="0" t="s">
+        <v>67</v>
+      </c>
+      <c r="D14" s="0" t="s">
+        <v>50</v>
+      </c>
+      <c r="E14" s="0" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C15" s="0" t="s">
+        <v>69</v>
+      </c>
+      <c r="D15" s="0" t="s">
+        <v>50</v>
+      </c>
+      <c r="E15" s="0" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="B16" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C16" s="0" t="s">
+        <v>71</v>
+      </c>
+      <c r="D16" s="0" t="s">
+        <v>50</v>
+      </c>
+      <c r="E16" s="0" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="B17" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C17" s="0" t="s">
+        <v>73</v>
+      </c>
+      <c r="D17" s="0" t="s">
+        <v>50</v>
+      </c>
+      <c r="E17" s="0" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="B18" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C18" s="0" t="s">
+        <v>75</v>
+      </c>
+      <c r="D18" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="E18" s="0" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="B19" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C19" s="0" t="s">
+        <v>77</v>
+      </c>
+      <c r="D19" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="E19" s="0" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="B20" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C20" s="0" t="s">
+        <v>79</v>
+      </c>
+      <c r="D20" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="E20" s="0" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="B21" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C21" s="0" t="s">
+        <v>81</v>
+      </c>
+      <c r="D21" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="E21" s="0" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="B22" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C22" s="0" t="s">
+        <v>83</v>
+      </c>
+      <c r="D22" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="E22" s="0" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="B23" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C23" s="0" t="s">
+        <v>85</v>
+      </c>
+      <c r="D23" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="E23" s="0" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="B24" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C24" s="0" t="s">
+        <v>87</v>
+      </c>
+      <c r="D24" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="E24" s="0" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="B25" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C25" s="0" t="s">
+        <v>89</v>
+      </c>
+      <c r="D25" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="E25" s="0" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="B26" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C26" s="0" t="s">
+        <v>91</v>
+      </c>
+      <c r="D26" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="E26" s="0" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="B27" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C27" s="0" t="s">
+        <v>93</v>
+      </c>
+      <c r="D27" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="E27" s="0" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="B28" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C28" s="0" t="s">
+        <v>95</v>
+      </c>
+      <c r="D28" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="E28" s="0" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="B29" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C29" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="D29" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="E29" s="0" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="B30" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C30" s="0" t="s">
+        <v>99</v>
+      </c>
+      <c r="D30" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="E30" s="0" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="B31" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C31" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="D31" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="E31" s="0" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="B32" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C32" s="0" t="s">
+        <v>103</v>
+      </c>
+      <c r="D32" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="E32" s="0" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="B33" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C33" s="0" t="s">
+        <v>105</v>
+      </c>
+      <c r="D33" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="E33" s="0" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="B34" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C34" s="0" t="s">
+        <v>107</v>
+      </c>
+      <c r="D34" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="E34" s="0" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="B35" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C35" s="0" t="s">
+        <v>109</v>
+      </c>
+      <c r="D35" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="E35" s="0" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="B36" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C36" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="D36" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="E36" s="0" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="B37" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C37" s="0" t="s">
+        <v>113</v>
+      </c>
+      <c r="D37" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="E37" s="0" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="B38" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C38" s="0" t="s">
+        <v>115</v>
+      </c>
+      <c r="D38" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="E38" s="0" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="1" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>